<commit_message>
Update Calc_Weighted_Average.xlsx for enhanced data analysis
</commit_message>
<xml_diff>
--- a/Calc_Weighted_Average.xlsx
+++ b/Calc_Weighted_Average.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Si24\root_scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27386279-4E0D-4AD0-9271-D961F3BD5FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D3AD6A3-506D-4029-B830-FA61404EEE21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5616" yWindow="312" windowWidth="17280" windowHeight="9072" xr2:uid="{49128516-656E-4F2E-B8C4-C265BEB2B077}"/>
   </bookViews>
@@ -673,17 +673,10 @@
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
-    <numFmt numFmtId="167" formatCode="0.00_ "/>
-    <numFmt numFmtId="169" formatCode="0.00000"/>
+    <numFmt numFmtId="166" formatCode="0.00_ "/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -781,26 +774,26 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -809,46 +802,46 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1865,7 +1858,7 @@
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="6">
-        <f t="shared" si="4"/>
+        <f>(C16-C$17)^2*E16</f>
         <v>3.700431820642736</v>
       </c>
       <c r="I16" s="6"/>
@@ -1940,7 +1933,7 @@
       <c r="K18" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="11" type="noConversion"/>
+  <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Calc_Weighted_Average.xlsx for improved data analysis
</commit_message>
<xml_diff>
--- a/Calc_Weighted_Average.xlsx
+++ b/Calc_Weighted_Average.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Si24\root_scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D3AD6A3-506D-4029-B830-FA61404EEE21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F35677-DAF0-483B-A43E-A2F96D3DC4F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5616" yWindow="312" windowWidth="17280" windowHeight="9072" xr2:uid="{49128516-656E-4F2E-B8C4-C265BEB2B077}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{49128516-656E-4F2E-B8C4-C265BEB2B077}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
   <si>
     <r>
       <t>a</t>
@@ -664,6 +664,18 @@
   </si>
   <si>
     <t>χ2/(n-1)</t>
+  </si>
+  <si>
+    <t>Degrees of Freedom</t>
+  </si>
+  <si>
+    <t>Critical Reduced χ2 (99% CI)</t>
+  </si>
+  <si>
+    <t>Inflation</t>
+  </si>
+  <si>
+    <t>Factor</t>
   </si>
 </sst>
 </file>
@@ -776,7 +788,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -823,9 +835,6 @@
     <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -842,6 +851,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1159,7 +1183,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C1CB840-A9D2-4CDC-90F2-19E028D0F72E}">
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" style="7" bestFit="1" customWidth="1"/>
@@ -1176,10 +1200,13 @@
     <col min="13" max="13" width="6.109375" style="7" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.6640625" style="7" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="19.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="7"/>
+    <col min="16" max="18" width="8.88671875" style="7"/>
+    <col min="19" max="19" width="17.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="23.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="8.88671875" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="9" t="s">
@@ -1206,7 +1233,7 @@
       <c r="J1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="K1" s="17" t="s">
         <v>14</v>
       </c>
       <c r="M1" s="7" t="s">
@@ -1218,17 +1245,23 @@
       <c r="O1" s="7" t="s">
         <v>17</v>
       </c>
+      <c r="S1" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="T1" s="7" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="22">
+      <c r="C2" s="21">
         <f>M2</f>
         <v>62</v>
       </c>
-      <c r="D2" s="22">
+      <c r="D2" s="21">
         <f>N2</f>
         <v>3</v>
       </c>
@@ -1249,7 +1282,7 @@
       <c r="J2" s="1">
         <v>0</v>
       </c>
-      <c r="K2" s="21">
+      <c r="K2" s="20">
         <f>F2/F$17</f>
         <v>2.0118329964132243E-4</v>
       </c>
@@ -1262,17 +1295,23 @@
       <c r="O2" s="7" t="s">
         <v>18</v>
       </c>
+      <c r="S2" s="7">
+        <v>1</v>
+      </c>
+      <c r="T2" s="7">
+        <v>6.6349999999999998</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="22">
+      <c r="C3" s="21">
         <f t="shared" ref="C3:C16" si="0">M3</f>
         <v>63</v>
       </c>
-      <c r="D3" s="22">
+      <c r="D3" s="21">
         <f t="shared" ref="D3:D16" si="1">N3</f>
         <v>5</v>
       </c>
@@ -1286,14 +1325,14 @@
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="6">
-        <f t="shared" ref="H3:H16" si="4">(C3-C$17)^2*E3</f>
+        <f t="shared" ref="H3:H15" si="4">(C3-C$17)^2*E3</f>
         <v>0.958575893146702</v>
       </c>
       <c r="I3" s="6"/>
       <c r="J3" s="1">
         <v>1</v>
       </c>
-      <c r="K3" s="21">
+      <c r="K3" s="20">
         <f t="shared" ref="K3:K16" si="5">F3/F$17</f>
         <v>7.3594148965567638E-5</v>
       </c>
@@ -1306,17 +1345,23 @@
       <c r="O3" s="7" t="s">
         <v>19</v>
       </c>
+      <c r="S3" s="7">
+        <v>2</v>
+      </c>
+      <c r="T3" s="7">
+        <v>4.6050000000000004</v>
+      </c>
     </row>
-    <row r="4" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="22">
+      <c r="C4" s="21">
         <f t="shared" si="0"/>
         <v>63</v>
       </c>
-      <c r="D4" s="22">
+      <c r="D4" s="21">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
@@ -1337,7 +1382,7 @@
       <c r="J4" s="1">
         <v>2</v>
       </c>
-      <c r="K4" s="21">
+      <c r="K4" s="20">
         <f t="shared" si="5"/>
         <v>7.3594148965567638E-5</v>
       </c>
@@ -1350,17 +1395,23 @@
       <c r="O4" s="7" t="s">
         <v>20</v>
       </c>
+      <c r="S4" s="7">
+        <v>3</v>
+      </c>
+      <c r="T4" s="7">
+        <v>3.782</v>
+      </c>
     </row>
-    <row r="5" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="21">
         <f t="shared" si="0"/>
         <v>64.2</v>
       </c>
-      <c r="D5" s="22">
+      <c r="D5" s="21">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
@@ -1381,7 +1432,7 @@
       <c r="J5" s="1">
         <v>3</v>
       </c>
-      <c r="K5" s="21">
+      <c r="K5" s="20">
         <f t="shared" si="5"/>
         <v>4.6872463924498437E-4</v>
       </c>
@@ -1394,17 +1445,23 @@
       <c r="O5" s="7" t="s">
         <v>21</v>
       </c>
+      <c r="S5" s="7">
+        <v>4</v>
+      </c>
+      <c r="T5" s="7">
+        <v>3.319</v>
+      </c>
     </row>
-    <row r="6" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A6" s="13"/>
       <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="21">
         <f t="shared" si="0"/>
         <v>66.7</v>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="21">
         <f t="shared" si="1"/>
         <v>0.7</v>
       </c>
@@ -1425,7 +1482,7 @@
       <c r="J6" s="1">
         <v>4</v>
       </c>
-      <c r="K6" s="21">
+      <c r="K6" s="20">
         <f t="shared" si="5"/>
         <v>3.975323725302367E-3</v>
       </c>
@@ -1438,17 +1495,23 @@
       <c r="O6" s="7" t="s">
         <v>22</v>
       </c>
+      <c r="S6" s="7">
+        <v>5</v>
+      </c>
+      <c r="T6" s="7">
+        <v>3.0169999999999999</v>
+      </c>
     </row>
-    <row r="7" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A7" s="13"/>
       <c r="B7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="21">
         <f t="shared" si="0"/>
         <v>66.900000000000006</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="21">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
@@ -1469,7 +1532,7 @@
       <c r="J7" s="1">
         <v>5</v>
       </c>
-      <c r="K7" s="21">
+      <c r="K7" s="20">
         <f t="shared" si="5"/>
         <v>1.9537494308716173E-3</v>
       </c>
@@ -1482,17 +1545,23 @@
       <c r="O7" s="7" t="s">
         <v>23</v>
       </c>
+      <c r="S7" s="7">
+        <v>6</v>
+      </c>
+      <c r="T7" s="7">
+        <v>2.802</v>
+      </c>
     </row>
-    <row r="8" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
       <c r="B8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="21">
         <f t="shared" si="0"/>
         <v>67.8</v>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="21">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
@@ -1513,7 +1582,7 @@
       <c r="J8" s="1">
         <v>6</v>
       </c>
-      <c r="K8" s="21">
+      <c r="K8" s="20">
         <f t="shared" si="5"/>
         <v>1.9800330555021766E-3</v>
       </c>
@@ -1526,17 +1595,23 @@
       <c r="O8" s="7" t="s">
         <v>23</v>
       </c>
+      <c r="S8" s="7">
+        <v>7</v>
+      </c>
+      <c r="T8" s="7">
+        <v>2.6389999999999998</v>
+      </c>
     </row>
-    <row r="9" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A9" s="13"/>
       <c r="B9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="21">
         <f t="shared" si="0"/>
         <v>68.3</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="21">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
@@ -1557,7 +1632,7 @@
       <c r="J9" s="1">
         <v>7</v>
       </c>
-      <c r="K9" s="21">
+      <c r="K9" s="20">
         <f t="shared" si="5"/>
         <v>4.9865876729645521E-2</v>
       </c>
@@ -1570,17 +1645,23 @@
       <c r="O9" s="7" t="s">
         <v>24</v>
       </c>
+      <c r="S9" s="7">
+        <v>8</v>
+      </c>
+      <c r="T9" s="7">
+        <v>2.5110000000000001</v>
+      </c>
     </row>
-    <row r="10" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A10" s="13"/>
       <c r="B10" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="21">
         <f t="shared" si="0"/>
         <v>68.5</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="21">
         <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
@@ -1601,7 +1682,7 @@
       <c r="J10" s="1">
         <v>8</v>
       </c>
-      <c r="K10" s="21">
+      <c r="K10" s="20">
         <f t="shared" si="5"/>
         <v>1.2502974216620492E-2</v>
       </c>
@@ -1614,17 +1695,23 @@
       <c r="O10" s="7" t="s">
         <v>25</v>
       </c>
+      <c r="S10" s="7">
+        <v>9</v>
+      </c>
+      <c r="T10" s="7">
+        <v>2.407</v>
+      </c>
     </row>
-    <row r="11" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A11" s="13"/>
       <c r="B11" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="21">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="21">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
@@ -1645,7 +1732,7 @@
       <c r="J11" s="1">
         <v>9</v>
       </c>
-      <c r="K11" s="21">
+      <c r="K11" s="20">
         <f t="shared" si="5"/>
         <v>1.2776761973188824E-4</v>
       </c>
@@ -1658,17 +1745,23 @@
       <c r="O11" s="7" t="s">
         <v>26</v>
       </c>
+      <c r="S11" s="7">
+        <v>10</v>
+      </c>
+      <c r="T11" s="7">
+        <v>2.3210000000000002</v>
+      </c>
     </row>
-    <row r="12" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
       <c r="B12" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="21">
         <f t="shared" si="0"/>
         <v>67.7</v>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="21">
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
@@ -1689,7 +1782,7 @@
       <c r="J12" s="1">
         <v>10</v>
       </c>
-      <c r="K12" s="21">
+      <c r="K12" s="20">
         <f t="shared" si="5"/>
         <v>0.19771126527654476</v>
       </c>
@@ -1702,17 +1795,23 @@
       <c r="O12" s="7" t="s">
         <v>27</v>
       </c>
+      <c r="S12" s="7">
+        <v>11</v>
+      </c>
+      <c r="T12" s="7">
+        <v>2.2480000000000002</v>
+      </c>
     </row>
-    <row r="13" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A13" s="13"/>
       <c r="B13" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="21">
         <f t="shared" si="0"/>
         <v>67.599999999999994</v>
       </c>
-      <c r="D13" s="22">
+      <c r="D13" s="21">
         <f t="shared" si="1"/>
         <v>0.25</v>
       </c>
@@ -1733,7 +1832,7 @@
       <c r="J13" s="1">
         <v>11</v>
       </c>
-      <c r="K13" s="21">
+      <c r="K13" s="20">
         <f t="shared" si="5"/>
         <v>3.1587076000459506E-2</v>
       </c>
@@ -1746,17 +1845,23 @@
       <c r="O13" s="7" t="s">
         <v>28</v>
       </c>
+      <c r="S13" s="7">
+        <v>12</v>
+      </c>
+      <c r="T13" s="7">
+        <v>2.1850000000000001</v>
+      </c>
     </row>
-    <row r="14" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
       <c r="B14" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="21">
         <f t="shared" si="0"/>
         <v>67.86</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="21">
         <f t="shared" si="1"/>
         <v>0.09</v>
       </c>
@@ -1777,7 +1882,7 @@
       <c r="J14" s="1">
         <v>12</v>
       </c>
-      <c r="K14" s="21">
+      <c r="K14" s="20">
         <f t="shared" si="5"/>
         <v>0.24466485149928568</v>
       </c>
@@ -1790,17 +1895,23 @@
       <c r="O14" s="7" t="s">
         <v>29</v>
       </c>
+      <c r="S14" s="7">
+        <v>13</v>
+      </c>
+      <c r="T14" s="7">
+        <v>2.13</v>
+      </c>
     </row>
-    <row r="15" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>
       <c r="B15" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="22">
+      <c r="C15" s="21">
         <f t="shared" si="0"/>
         <v>67.599999999999994</v>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="21">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
@@ -1821,7 +1932,7 @@
       <c r="J15" s="1">
         <v>13</v>
       </c>
-      <c r="K15" s="21">
+      <c r="K15" s="20">
         <f t="shared" si="5"/>
         <v>4.9354806250717961E-2</v>
       </c>
@@ -1834,17 +1945,23 @@
       <c r="O15" s="7" t="s">
         <v>30</v>
       </c>
+      <c r="S15" s="7">
+        <v>14</v>
+      </c>
+      <c r="T15" s="7">
+        <v>2.0819999999999999</v>
+      </c>
     </row>
-    <row r="16" spans="1:15" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A16" s="13"/>
       <c r="B16" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="22">
+      <c r="C16" s="21">
         <f t="shared" si="0"/>
         <v>68.03</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="21">
         <f t="shared" si="1"/>
         <v>7.0000000000000007E-2</v>
       </c>
@@ -1865,7 +1982,7 @@
       <c r="J16" s="1">
         <v>14</v>
       </c>
-      <c r="K16" s="21">
+      <c r="K16" s="20">
         <f t="shared" si="5"/>
         <v>0.40545917995850062</v>
       </c>
@@ -1878,8 +1995,14 @@
       <c r="O16" s="7" t="s">
         <v>31</v>
       </c>
+      <c r="S16" s="7">
+        <v>15</v>
+      </c>
+      <c r="T16" s="7">
+        <v>2.0390000000000001</v>
+      </c>
     </row>
-    <row r="17" spans="1:11" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A17" s="14"/>
       <c r="B17" s="2" t="s">
         <v>13</v>
@@ -1900,15 +2023,15 @@
         <f>SUM(F2:F16)</f>
         <v>34241.852585034008</v>
       </c>
-      <c r="G17" s="20">
+      <c r="G17" s="19">
         <f>SQRT(1/E17)</f>
         <v>4.452883894244377E-2</v>
       </c>
-      <c r="H17" s="16">
+      <c r="H17" s="25">
         <f>SUM(H2:H16)</f>
         <v>31.011057781641497</v>
       </c>
-      <c r="I17" s="20">
+      <c r="I17" s="19">
         <f>SQRT(H17/(J16*E17))</f>
         <v>6.6272849422103902E-2</v>
       </c>
@@ -1916,21 +2039,67 @@
         <f>H17/J16</f>
         <v>2.2150755558315356</v>
       </c>
-      <c r="K17" s="17"/>
+      <c r="K17" s="16"/>
+      <c r="S17" s="7">
+        <v>16</v>
+      </c>
+      <c r="T17" s="22">
+        <v>2</v>
+      </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="19"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="18"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="11" t="s">
+      <c r="J18" s="24" t="s">
         <v>42</v>
       </c>
       <c r="K18" s="1"/>
+      <c r="S18" s="7">
+        <v>17</v>
+      </c>
+      <c r="T18" s="7">
+        <v>1.9650000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="J19" s="23">
+        <f>SQRT(J17)</f>
+        <v>1.4883129898752936</v>
+      </c>
+      <c r="S19" s="7">
+        <v>18</v>
+      </c>
+      <c r="T19" s="7">
+        <v>1.9339999999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="J20" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="S20" s="7">
+        <v>19</v>
+      </c>
+      <c r="T20" s="7">
+        <v>1.905</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="J21" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="S21" s="7">
+        <v>20</v>
+      </c>
+      <c r="T21" s="7">
+        <v>1.8779999999999999</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="10" type="noConversion"/>

</xml_diff>